<commit_message>
City index 26-08 T2 wrap up
</commit_message>
<xml_diff>
--- a/data_indexpoints_tidy/tallmateriale_19954.xlsx
+++ b/data_indexpoints_tidy/tallmateriale_19954.xlsx
@@ -9,16 +9,17 @@
   <sheets>
     <sheet name="punkt_adt" sheetId="1" r:id="rId1"/>
     <sheet name="punktindeks_maned" sheetId="2" r:id="rId2"/>
-    <sheet name="byindeks_aarlig" sheetId="3" r:id="rId3"/>
-    <sheet name="byindeks_hittil" sheetId="4" r:id="rId4"/>
-    <sheet name="by_glid_indeks" sheetId="5" r:id="rId5"/>
+    <sheet name="punktindeks_aar" sheetId="3" r:id="rId3"/>
+    <sheet name="byindeks_aarlig" sheetId="4" r:id="rId4"/>
+    <sheet name="byindeks_hittil" sheetId="5" r:id="rId5"/>
+    <sheet name="by_glid_indeks" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="115">
   <si>
     <t>trp_id</t>
   </si>
@@ -248,6 +249,12 @@
     <t>des</t>
   </si>
   <si>
+    <t>index_2024_2025</t>
+  </si>
+  <si>
+    <t>index_2025_2026</t>
+  </si>
+  <si>
     <t>area_name</t>
   </si>
   <si>
@@ -299,7 +306,7 @@
     <t>2025-2026</t>
   </si>
   <si>
-    <t>jan-jul</t>
+    <t>jan-aug</t>
   </si>
   <si>
     <t>2024-2026</t>
@@ -354,6 +361,9 @@
   </si>
   <si>
     <t>2024 - (aug 2025 - jul 2026)</t>
+  </si>
+  <si>
+    <t>2024 - (sep 2025 - aug 2026)</t>
   </si>
 </sst>
 </file>
@@ -1405,6 +1415,9 @@
       <c r="K3">
         <v>-2.26</v>
       </c>
+      <c r="L3">
+        <v>-0.17</v>
+      </c>
     </row>
     <row r="4" spans="1:16">
       <c r="A4" t="s">
@@ -1481,6 +1494,9 @@
       <c r="K5">
         <v>-2.17</v>
       </c>
+      <c r="L5">
+        <v>0.57</v>
+      </c>
     </row>
     <row r="6" spans="1:16">
       <c r="A6" t="s">
@@ -1566,6 +1582,9 @@
       <c r="K7">
         <v>-3.28</v>
       </c>
+      <c r="L7">
+        <v>0.31</v>
+      </c>
     </row>
     <row r="8" spans="1:16">
       <c r="A8" t="s">
@@ -1639,6 +1658,9 @@
       <c r="K9">
         <v>-12.55</v>
       </c>
+      <c r="L9">
+        <v>-3.92</v>
+      </c>
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
@@ -1724,6 +1746,9 @@
       <c r="K11">
         <v>-5.95</v>
       </c>
+      <c r="L11">
+        <v>3.19</v>
+      </c>
     </row>
     <row r="12" spans="1:16">
       <c r="A12" t="s">
@@ -1809,6 +1834,9 @@
       <c r="K13">
         <v>-5.39</v>
       </c>
+      <c r="L13">
+        <v>0.02</v>
+      </c>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" t="s">
@@ -1894,6 +1922,9 @@
       <c r="K15">
         <v>9.75</v>
       </c>
+      <c r="L15">
+        <v>7.65</v>
+      </c>
     </row>
     <row r="16" spans="1:16">
       <c r="A16" t="s">
@@ -1979,6 +2010,9 @@
       <c r="K17">
         <v>2.77</v>
       </c>
+      <c r="L17">
+        <v>3.31</v>
+      </c>
     </row>
     <row r="18" spans="1:16">
       <c r="A18" t="s">
@@ -2062,7 +2096,7 @@
         <v>2.96</v>
       </c>
       <c r="K19">
-        <v>-7.43</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="20" spans="1:16">
@@ -2200,6 +2234,9 @@
       </c>
       <c r="K23">
         <v>-4.08</v>
+      </c>
+      <c r="L23">
+        <v>-0.32</v>
       </c>
     </row>
   </sheetData>
@@ -2209,139 +2246,208 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1">
+    <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2">
-        <v>2024</v>
-      </c>
-      <c r="C2">
-        <v>2025</v>
-      </c>
-      <c r="D2" t="s">
-        <v>89</v>
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2">
+        <v>1.54</v>
       </c>
       <c r="E2">
-        <v>12</v>
-      </c>
-      <c r="F2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H2" t="s">
-        <v>91</v>
-      </c>
-      <c r="I2">
-        <v>11</v>
-      </c>
-      <c r="J2">
-        <v>1.0224</v>
-      </c>
-      <c r="K2">
-        <v>2.24</v>
-      </c>
-      <c r="L2">
-        <v>1.599862085038858</v>
-      </c>
-      <c r="M2">
-        <v>-0.9</v>
-      </c>
-      <c r="N2">
-        <v>5.38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3">
-        <v>2025</v>
-      </c>
-      <c r="C3">
-        <v>2026</v>
-      </c>
-      <c r="D3" t="s">
-        <v>92</v>
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3">
+        <v>0.43</v>
       </c>
       <c r="E3">
-        <v>7</v>
-      </c>
-      <c r="F3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G3" t="s">
-        <v>93</v>
-      </c>
-      <c r="H3" t="s">
-        <v>91</v>
-      </c>
-      <c r="I3">
-        <v>10</v>
-      </c>
-      <c r="J3">
-        <v>1.0188</v>
-      </c>
-      <c r="K3">
-        <v>1.88</v>
-      </c>
-      <c r="L3">
-        <v>0.869684112228528</v>
-      </c>
-      <c r="M3">
-        <v>0.18</v>
-      </c>
-      <c r="N3">
-        <v>3.58</v>
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4">
+        <v>1.66</v>
+      </c>
+      <c r="E4">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5">
+        <v>12.06</v>
+      </c>
+      <c r="E5">
+        <v>-2.74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6">
+        <v>-4.52</v>
+      </c>
+      <c r="E6">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7">
+        <v>3.73</v>
+      </c>
+      <c r="E7">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8">
+        <v>0.17</v>
+      </c>
+      <c r="E8">
+        <v>6.07</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9">
+        <v>7.14</v>
+      </c>
+      <c r="E9">
+        <v>5.09</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10">
+        <v>6.33</v>
+      </c>
+      <c r="E10">
+        <v>4.34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11">
+        <v>-8.33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12">
+        <v>-1.2</v>
+      </c>
+      <c r="E12">
+        <v>-2.03</v>
       </c>
     </row>
   </sheetData>
@@ -2351,51 +2457,51 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:14" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -2409,37 +2515,37 @@
         <v>2025</v>
       </c>
       <c r="D2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E2">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H2" t="s">
         <v>93</v>
-      </c>
-      <c r="H2" t="s">
-        <v>91</v>
       </c>
       <c r="I2">
         <v>11</v>
       </c>
       <c r="J2">
-        <v>1.0149</v>
+        <v>1.0224</v>
       </c>
       <c r="K2">
-        <v>1.49</v>
+        <v>2.24</v>
       </c>
       <c r="L2">
-        <v>1.323998280676608</v>
+        <v>1.599862085038858</v>
       </c>
       <c r="M2">
-        <v>-1.11</v>
+        <v>-0.9</v>
       </c>
       <c r="N2">
-        <v>4.09</v>
+        <v>5.38</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -2453,19 +2559,19 @@
         <v>2026</v>
       </c>
       <c r="D3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G3" t="s">
+        <v>95</v>
+      </c>
+      <c r="H3" t="s">
         <v>93</v>
-      </c>
-      <c r="H3" t="s">
-        <v>91</v>
       </c>
       <c r="I3">
         <v>10</v>
@@ -2477,57 +2583,13 @@
         <v>1.88</v>
       </c>
       <c r="L3">
-        <v>0.869684112228528</v>
+        <v>0.8914653979552348</v>
       </c>
       <c r="M3">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
       <c r="N3">
-        <v>3.58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4">
-        <v>2024</v>
-      </c>
-      <c r="C4">
-        <v>2026</v>
-      </c>
-      <c r="D4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E4">
-        <v>7</v>
-      </c>
-      <c r="F4" t="s">
-        <v>70</v>
-      </c>
-      <c r="G4" t="s">
-        <v>93</v>
-      </c>
-      <c r="H4" t="s">
-        <v>95</v>
-      </c>
-      <c r="I4">
-        <v>11</v>
-      </c>
-      <c r="J4">
-        <v>1.034</v>
-      </c>
-      <c r="K4">
-        <v>3.4</v>
-      </c>
-      <c r="L4">
-        <v>1.612046198451599</v>
-      </c>
-      <c r="M4">
-        <v>0.24</v>
-      </c>
-      <c r="N4">
-        <v>6.56</v>
+        <v>3.63</v>
       </c>
     </row>
   </sheetData>
@@ -2537,7 +2599,193 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:14" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2">
+        <v>2024</v>
+      </c>
+      <c r="C2">
+        <v>2025</v>
+      </c>
+      <c r="D2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E2">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H2" t="s">
+        <v>93</v>
+      </c>
+      <c r="I2">
+        <v>11</v>
+      </c>
+      <c r="J2">
+        <v>1.0178</v>
+      </c>
+      <c r="K2">
+        <v>1.78</v>
+      </c>
+      <c r="L2">
+        <v>1.410802235780169</v>
+      </c>
+      <c r="M2">
+        <v>-0.99</v>
+      </c>
+      <c r="N2">
+        <v>4.55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3">
+        <v>2025</v>
+      </c>
+      <c r="C3">
+        <v>2026</v>
+      </c>
+      <c r="D3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G3" t="s">
+        <v>95</v>
+      </c>
+      <c r="H3" t="s">
+        <v>93</v>
+      </c>
+      <c r="I3">
+        <v>10</v>
+      </c>
+      <c r="J3">
+        <v>1.0188</v>
+      </c>
+      <c r="K3">
+        <v>1.88</v>
+      </c>
+      <c r="L3">
+        <v>0.8914653979552348</v>
+      </c>
+      <c r="M3">
+        <v>0.13</v>
+      </c>
+      <c r="N3">
+        <v>3.63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <v>2024</v>
+      </c>
+      <c r="C4">
+        <v>2026</v>
+      </c>
+      <c r="D4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G4" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" t="s">
+        <v>97</v>
+      </c>
+      <c r="I4">
+        <v>11</v>
+      </c>
+      <c r="J4">
+        <v>1.0369</v>
+      </c>
+      <c r="K4">
+        <v>3.69</v>
+      </c>
+      <c r="L4">
+        <v>1.699798897840267</v>
+      </c>
+      <c r="M4">
+        <v>0.36</v>
+      </c>
+      <c r="N4">
+        <v>7.02</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="20.7109375" style="2" customWidth="1"/>
@@ -2548,40 +2796,40 @@
         <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="K1" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -2595,10 +2843,10 @@
         <v>45992</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F2">
         <v>1.0335</v>
@@ -2636,10 +2884,10 @@
         <v>46023</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F3">
         <v>1.0357</v>
@@ -2677,10 +2925,10 @@
         <v>46054</v>
       </c>
       <c r="D4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F4">
         <v>1.0388</v>
@@ -2718,10 +2966,10 @@
         <v>46082</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F5">
         <v>1.0426</v>
@@ -2759,10 +3007,10 @@
         <v>46113</v>
       </c>
       <c r="D6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F6">
         <v>1.0481</v>
@@ -2800,10 +3048,10 @@
         <v>46143</v>
       </c>
       <c r="D7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F7">
         <v>1.0482</v>
@@ -2841,10 +3089,10 @@
         <v>46174</v>
       </c>
       <c r="D8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F8">
         <v>1.0505</v>
@@ -2882,22 +3130,22 @@
         <v>46204</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F9">
-        <v>1.0484</v>
+        <v>1.0491</v>
       </c>
       <c r="G9">
-        <v>4.84</v>
+        <v>4.91</v>
       </c>
       <c r="H9">
         <v>1.4</v>
       </c>
       <c r="I9">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="J9">
         <v>8</v>
@@ -2906,10 +3154,51 @@
         <v>7</v>
       </c>
       <c r="L9">
-        <v>3.82</v>
+        <v>3.91</v>
       </c>
       <c r="M9">
-        <v>1.45</v>
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10">
+        <v>2026</v>
+      </c>
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2">
+        <v>46235</v>
+      </c>
+      <c r="D10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E10" t="s">
+        <v>114</v>
+      </c>
+      <c r="F10">
+        <v>1.0501</v>
+      </c>
+      <c r="G10">
+        <v>5.01</v>
+      </c>
+      <c r="H10">
+        <v>1.5</v>
+      </c>
+      <c r="I10">
+        <v>8.5</v>
+      </c>
+      <c r="J10">
+        <v>8</v>
+      </c>
+      <c r="K10">
+        <v>7</v>
+      </c>
+      <c r="L10">
+        <v>3.95</v>
+      </c>
+      <c r="M10">
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>